<commit_message>
resolve unusual n_projs value (8)
</commit_message>
<xml_diff>
--- a/data/raw/parcial_quali.xlsx
+++ b/data/raw/parcial_quali.xlsx
@@ -12972,10 +12972,8 @@
           <t>Junior (up to 5 years)</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>7-10, mostly university projects</t>
-        </is>
+      <c r="I43" t="n">
+        <v>8</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>

</xml_diff>